<commit_message>
nuovo metodo di eseguire le simulazioni
le eseguiamo tutte e 70 e mettiamo su un grafico l'andamento di come trova i fault
</commit_message>
<xml_diff>
--- a/LaneFollowingControlWithSensorFusionAndLaneDetectionExample/tabellarisultatiHecate_CONF1.xlsx
+++ b/LaneFollowingControlWithSensorFusionAndLaneDetectionExample/tabellarisultatiHecate_CONF1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="85" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="241" uniqueCount="22">
   <si>
     <t>Scenario</t>
   </si>
@@ -70,6 +70,15 @@
   </si>
   <si>
     <t>Total_Fault_Found</t>
+  </si>
+  <si>
+    <t>Highway_double_target</t>
+  </si>
+  <si>
+    <t>curvaLunga</t>
+  </si>
+  <si>
+    <t>ACC_01_ISO_TargetDiscriminationTest</t>
   </si>
 </sst>
 </file>
@@ -156,7 +165,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="0">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -745,21 +754,29 @@
       <c r="E41" s="0"/>
     </row>
     <row r="42">
-      <c r="A42" s="0"/>
-      <c r="B42" s="0"/>
+      <c r="A42" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>13</v>
+      </c>
       <c r="C42" s="0">
-        <v>0</v>
+        <v>-4.9132709455110097</v>
       </c>
       <c r="D42" s="0" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" s="0"/>
     </row>
     <row r="43">
-      <c r="A43" s="0"/>
-      <c r="B43" s="0"/>
+      <c r="A43" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B43" s="0" t="s">
+        <v>10</v>
+      </c>
       <c r="C43" s="0">
-        <v>0</v>
+        <v>23.343334587647796</v>
       </c>
       <c r="D43" s="0" t="b">
         <v>0</v>
@@ -767,10 +784,14 @@
       <c r="E43" s="0"/>
     </row>
     <row r="44">
-      <c r="A44" s="0"/>
-      <c r="B44" s="0"/>
+      <c r="A44" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="C44" s="0">
-        <v>0</v>
+        <v>1.9506559854166206</v>
       </c>
       <c r="D44" s="0" t="b">
         <v>0</v>
@@ -778,10 +799,14 @@
       <c r="E44" s="0"/>
     </row>
     <row r="45">
-      <c r="A45" s="0"/>
-      <c r="B45" s="0"/>
+      <c r="A45" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>11</v>
+      </c>
       <c r="C45" s="0">
-        <v>0</v>
+        <v>21.209269994395491</v>
       </c>
       <c r="D45" s="0" t="b">
         <v>0</v>
@@ -789,65 +814,89 @@
       <c r="E45" s="0"/>
     </row>
     <row r="46">
-      <c r="A46" s="0"/>
-      <c r="B46" s="0"/>
+      <c r="A46" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B46" s="0" t="s">
+        <v>11</v>
+      </c>
       <c r="C46" s="0">
-        <v>0</v>
+        <v>-4.9637324106799197</v>
       </c>
       <c r="D46" s="0" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="0"/>
     </row>
     <row r="47">
-      <c r="A47" s="0"/>
-      <c r="B47" s="0"/>
+      <c r="A47" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>14</v>
+      </c>
       <c r="C47" s="0">
-        <v>0</v>
+        <v>-5.0485200940389836</v>
       </c>
       <c r="D47" s="0" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" s="0"/>
     </row>
     <row r="48">
-      <c r="A48" s="0"/>
-      <c r="B48" s="0"/>
+      <c r="A48" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" s="0" t="s">
+        <v>9</v>
+      </c>
       <c r="C48" s="0">
-        <v>0</v>
+        <v>-5.1155456861083568</v>
       </c>
       <c r="D48" s="0" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" s="0"/>
     </row>
     <row r="49">
-      <c r="A49" s="0"/>
-      <c r="B49" s="0"/>
+      <c r="A49" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B49" s="0" t="s">
+        <v>13</v>
+      </c>
       <c r="C49" s="0">
-        <v>0</v>
+        <v>-5.0054774643551463</v>
       </c>
       <c r="D49" s="0" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" s="0"/>
     </row>
     <row r="50">
-      <c r="A50" s="0"/>
-      <c r="B50" s="0"/>
+      <c r="A50" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B50" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="C50" s="0">
-        <v>0</v>
+        <v>-4.8224758114685278</v>
       </c>
       <c r="D50" s="0" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" s="0"/>
     </row>
     <row r="51">
-      <c r="A51" s="0"/>
-      <c r="B51" s="0"/>
+      <c r="A51" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B51" s="0" t="s">
+        <v>13</v>
+      </c>
       <c r="C51" s="0">
-        <v>0</v>
+        <v>-5.7460253769178946</v>
       </c>
       <c r="D51" s="0" t="b">
         <v>0</v>
@@ -855,10 +904,14 @@
       <c r="E51" s="0"/>
     </row>
     <row r="52">
-      <c r="A52" s="0"/>
-      <c r="B52" s="0"/>
+      <c r="A52" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="0" t="s">
+        <v>14</v>
+      </c>
       <c r="C52" s="0">
-        <v>0</v>
+        <v>28.874252804143765</v>
       </c>
       <c r="D52" s="0" t="b">
         <v>0</v>
@@ -866,10 +919,14 @@
       <c r="E52" s="0"/>
     </row>
     <row r="53">
-      <c r="A53" s="0"/>
-      <c r="B53" s="0"/>
+      <c r="A53" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B53" s="0" t="s">
+        <v>13</v>
+      </c>
       <c r="C53" s="0">
-        <v>0</v>
+        <v>24.063587591923785</v>
       </c>
       <c r="D53" s="0" t="b">
         <v>0</v>
@@ -877,10 +934,14 @@
       <c r="E53" s="0"/>
     </row>
     <row r="54">
-      <c r="A54" s="0"/>
-      <c r="B54" s="0"/>
+      <c r="A54" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>11</v>
+      </c>
       <c r="C54" s="0">
-        <v>0</v>
+        <v>29.91667766430195</v>
       </c>
       <c r="D54" s="0" t="b">
         <v>0</v>
@@ -888,10 +949,14 @@
       <c r="E54" s="0"/>
     </row>
     <row r="55">
-      <c r="A55" s="0"/>
-      <c r="B55" s="0"/>
+      <c r="A55" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>9</v>
+      </c>
       <c r="C55" s="0">
-        <v>0</v>
+        <v>29.592585200397785</v>
       </c>
       <c r="D55" s="0" t="b">
         <v>0</v>
@@ -899,10 +964,14 @@
       <c r="E55" s="0"/>
     </row>
     <row r="56">
-      <c r="A56" s="0"/>
-      <c r="B56" s="0"/>
+      <c r="A56" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="C56" s="0">
-        <v>0</v>
+        <v>29.948238707703801</v>
       </c>
       <c r="D56" s="0" t="b">
         <v>0</v>
@@ -910,10 +979,14 @@
       <c r="E56" s="0"/>
     </row>
     <row r="57">
-      <c r="A57" s="0"/>
-      <c r="B57" s="0"/>
+      <c r="A57" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B57" s="0" t="s">
+        <v>10</v>
+      </c>
       <c r="C57" s="0">
-        <v>0</v>
+        <v>30.055009820698551</v>
       </c>
       <c r="D57" s="0" t="b">
         <v>0</v>
@@ -921,10 +994,14 @@
       <c r="E57" s="0"/>
     </row>
     <row r="58">
-      <c r="A58" s="0"/>
-      <c r="B58" s="0"/>
+      <c r="A58" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" s="0" t="s">
+        <v>15</v>
+      </c>
       <c r="C58" s="0">
-        <v>0</v>
+        <v>30.174186611542254</v>
       </c>
       <c r="D58" s="0" t="b">
         <v>0</v>
@@ -932,10 +1009,14 @@
       <c r="E58" s="0"/>
     </row>
     <row r="59">
-      <c r="A59" s="0"/>
-      <c r="B59" s="0"/>
+      <c r="A59" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B59" s="0" t="s">
+        <v>11</v>
+      </c>
       <c r="C59" s="0">
-        <v>0</v>
+        <v>0.70527010787779609</v>
       </c>
       <c r="D59" s="0" t="b">
         <v>0</v>
@@ -943,10 +1024,14 @@
       <c r="E59" s="0"/>
     </row>
     <row r="60">
-      <c r="A60" s="0"/>
-      <c r="B60" s="0"/>
+      <c r="A60" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B60" s="0" t="s">
+        <v>14</v>
+      </c>
       <c r="C60" s="0">
-        <v>0</v>
+        <v>1.2624213627403336</v>
       </c>
       <c r="D60" s="0" t="b">
         <v>0</v>
@@ -954,10 +1039,14 @@
       <c r="E60" s="0"/>
     </row>
     <row r="61">
-      <c r="A61" s="0"/>
-      <c r="B61" s="0"/>
+      <c r="A61" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B61" s="0" t="s">
+        <v>15</v>
+      </c>
       <c r="C61" s="0">
-        <v>0</v>
+        <v>1.4772436234657196</v>
       </c>
       <c r="D61" s="0" t="b">
         <v>0</v>
@@ -965,10 +1054,14 @@
       <c r="E61" s="0"/>
     </row>
     <row r="62">
-      <c r="A62" s="0"/>
-      <c r="B62" s="0"/>
+      <c r="A62" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B62" s="0" t="s">
+        <v>9</v>
+      </c>
       <c r="C62" s="0">
-        <v>0</v>
+        <v>2.4264451165355911</v>
       </c>
       <c r="D62" s="0" t="b">
         <v>0</v>
@@ -976,10 +1069,14 @@
       <c r="E62" s="0"/>
     </row>
     <row r="63">
-      <c r="A63" s="0"/>
-      <c r="B63" s="0"/>
+      <c r="A63" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B63" s="0" t="s">
+        <v>10</v>
+      </c>
       <c r="C63" s="0">
-        <v>0</v>
+        <v>3.090034130685293</v>
       </c>
       <c r="D63" s="0" t="b">
         <v>0</v>
@@ -987,10 +1084,14 @@
       <c r="E63" s="0"/>
     </row>
     <row r="64">
-      <c r="A64" s="0"/>
-      <c r="B64" s="0"/>
+      <c r="A64" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B64" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="C64" s="0">
-        <v>0</v>
+        <v>3.5491290917359901</v>
       </c>
       <c r="D64" s="0" t="b">
         <v>0</v>
@@ -998,10 +1099,14 @@
       <c r="E64" s="0"/>
     </row>
     <row r="65">
-      <c r="A65" s="0"/>
-      <c r="B65" s="0"/>
+      <c r="A65" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B65" s="0" t="s">
+        <v>15</v>
+      </c>
       <c r="C65" s="0">
-        <v>0</v>
+        <v>37.094292868652857</v>
       </c>
       <c r="D65" s="0" t="b">
         <v>0</v>
@@ -1009,10 +1114,14 @@
       <c r="E65" s="0"/>
     </row>
     <row r="66">
-      <c r="A66" s="0"/>
-      <c r="B66" s="0"/>
+      <c r="A66" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B66" s="0" t="s">
+        <v>13</v>
+      </c>
       <c r="C66" s="0">
-        <v>0</v>
+        <v>37.105685164052545</v>
       </c>
       <c r="D66" s="0" t="b">
         <v>0</v>
@@ -1020,10 +1129,14 @@
       <c r="E66" s="0"/>
     </row>
     <row r="67">
-      <c r="A67" s="0"/>
-      <c r="B67" s="0"/>
+      <c r="A67" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B67" s="0" t="s">
+        <v>11</v>
+      </c>
       <c r="C67" s="0">
-        <v>0</v>
+        <v>38.224737862406691</v>
       </c>
       <c r="D67" s="0" t="b">
         <v>0</v>
@@ -1031,10 +1144,14 @@
       <c r="E67" s="0"/>
     </row>
     <row r="68">
-      <c r="A68" s="0"/>
-      <c r="B68" s="0"/>
+      <c r="A68" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B68" s="0" t="s">
+        <v>9</v>
+      </c>
       <c r="C68" s="0">
-        <v>0</v>
+        <v>38.515121907499733</v>
       </c>
       <c r="D68" s="0" t="b">
         <v>0</v>
@@ -1042,10 +1159,14 @@
       <c r="E68" s="0"/>
     </row>
     <row r="69">
-      <c r="A69" s="0"/>
-      <c r="B69" s="0"/>
+      <c r="A69" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B69" s="0" t="s">
+        <v>14</v>
+      </c>
       <c r="C69" s="0">
-        <v>0</v>
+        <v>38.652954511366083</v>
       </c>
       <c r="D69" s="0" t="b">
         <v>0</v>
@@ -1053,10 +1174,14 @@
       <c r="E69" s="0"/>
     </row>
     <row r="70">
-      <c r="A70" s="0"/>
-      <c r="B70" s="0"/>
+      <c r="A70" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B70" s="0" t="s">
+        <v>10</v>
+      </c>
       <c r="C70" s="0">
-        <v>0</v>
+        <v>38.413814022374339</v>
       </c>
       <c r="D70" s="0" t="b">
         <v>0</v>
@@ -1064,10 +1189,14 @@
       <c r="E70" s="0"/>
     </row>
     <row r="71">
-      <c r="A71" s="0"/>
-      <c r="B71" s="0"/>
+      <c r="A71" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B71" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="C71" s="0">
-        <v>0</v>
+        <v>38.52506278830694</v>
       </c>
       <c r="D71" s="0" t="b">
         <v>0</v>

</xml_diff>